<commit_message>
fix(cdpgf): export .xlsx via gabarit PizZip (corrige crash ExcelJS 'anchors')
ExcelJS plantait a la reecriture du gabarit contenant le logo (reading 'anchors').
Remplacement par une approche PizZip : on substitue uniquement le texte des
cellules (placeholders {{...}}), le logo et la mise en forme du gabarit ne sont
jamais retouches.
</commit_message>
<xml_diff>
--- a/backend/templates/CDPGF_template.xlsx
+++ b/backend/templates/CDPGF_template.xlsx
@@ -766,9 +766,7 @@
     <row r="6" ht="39" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOGEMENT LTS JAMALACS 3
-N° 20 RUE DES JAMALACS 
-</t>
+          <t>{{HEADER}}</t>
         </is>
       </c>
     </row>
@@ -842,194 +840,578 @@
       <c r="F10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>{{R1}}</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>{{DES1}}</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>{{U1}}</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>{{Q1}}</t>
+        </is>
+      </c>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>{{R2}}</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>{{DES2}}</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>{{U2}}</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>{{Q2}}</t>
+        </is>
+      </c>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>{{R3}}</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>{{DES3}}</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>{{U3}}</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>{{Q3}}</t>
+        </is>
+      </c>
       <c r="E13" s="11" t="n"/>
       <c r="F13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="15" t="n"/>
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>{{R4}}</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>{{DES4}}</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>{{U4}}</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>{{Q4}}</t>
+        </is>
+      </c>
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="11" t="n"/>
     </row>
     <row r="15" customFormat="1" s="4">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="15" t="n"/>
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>{{R5}}</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>{{DES5}}</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>{{U5}}</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>{{Q5}}</t>
+        </is>
+      </c>
       <c r="E15" s="11" t="n"/>
       <c r="F15" s="11" t="n"/>
     </row>
     <row r="16" customFormat="1" s="4">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>{{R6}}</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>{{DES6}}</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>{{U6}}</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>{{Q6}}</t>
+        </is>
+      </c>
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="11" t="n"/>
     </row>
     <row r="17" customFormat="1" s="4">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>{{R7}}</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>{{DES7}}</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>{{U7}}</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>{{Q7}}</t>
+        </is>
+      </c>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="15" t="n"/>
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>{{R8}}</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>{{DES8}}</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>{{U8}}</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>{{Q8}}</t>
+        </is>
+      </c>
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="14" t="n"/>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="15" t="n"/>
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>{{R9}}</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>{{DES9}}</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>{{U9}}</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>{{Q9}}</t>
+        </is>
+      </c>
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="15" t="n"/>
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>{{R10}}</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>{{DES10}}</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>{{U10}}</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>{{Q10}}</t>
+        </is>
+      </c>
       <c r="E20" s="11" t="n"/>
       <c r="F20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="15" t="n"/>
-      <c r="D21" s="15" t="n"/>
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>{{R11}}</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>{{DES11}}</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>{{U11}}</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>{{Q11}}</t>
+        </is>
+      </c>
       <c r="E21" s="11" t="n"/>
       <c r="F21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>{{R12}}</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>{{DES12}}</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>{{U12}}</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>{{Q12}}</t>
+        </is>
+      </c>
       <c r="E22" s="11" t="n"/>
       <c r="F22" s="11" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="15" t="n"/>
-      <c r="D23" s="15" t="n"/>
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>{{R13}}</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>{{DES13}}</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>{{U13}}</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>{{Q13}}</t>
+        </is>
+      </c>
       <c r="E23" s="11" t="n"/>
       <c r="F23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n"/>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>{{R14}}</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>{{DES14}}</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>{{U14}}</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>{{Q14}}</t>
+        </is>
+      </c>
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="11" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>{{R15}}</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>{{DES15}}</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>{{U15}}</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>{{Q15}}</t>
+        </is>
+      </c>
       <c r="E25" s="11" t="n"/>
       <c r="F25" s="11" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="n"/>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="15" t="n"/>
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>{{R16}}</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>{{DES16}}</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>{{U16}}</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>{{Q16}}</t>
+        </is>
+      </c>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="11" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n"/>
-      <c r="B27" s="14" t="n"/>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>{{R17}}</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>{{DES17}}</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>{{U17}}</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>{{Q17}}</t>
+        </is>
+      </c>
       <c r="E27" s="11" t="n"/>
       <c r="F27" s="11" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n"/>
-      <c r="B28" s="14" t="n"/>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>{{R18}}</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>{{DES18}}</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>{{U18}}</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>{{Q18}}</t>
+        </is>
+      </c>
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>{{R19}}</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>{{DES19}}</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>{{U19}}</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>{{Q19}}</t>
+        </is>
+      </c>
       <c r="E29" s="11" t="n"/>
       <c r="F29" s="11" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n"/>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="15" t="n"/>
-      <c r="D30" s="15" t="n"/>
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>{{R20}}</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>{{DES20}}</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>{{U20}}</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>{{Q20}}</t>
+        </is>
+      </c>
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>{{R21}}</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>{{DES21}}</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>{{U21}}</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>{{Q21}}</t>
+        </is>
+      </c>
       <c r="E31" s="11" t="n"/>
       <c r="F31" s="11" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="14" t="n"/>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>{{R22}}</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>{{DES22}}</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>{{U22}}</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>{{Q22}}</t>
+        </is>
+      </c>
       <c r="E32" s="11" t="n"/>
       <c r="F32" s="11" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>{{R23}}</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>{{DES23}}</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>{{U23}}</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>{{Q23}}</t>
+        </is>
+      </c>
       <c r="E33" s="11" t="n"/>
       <c r="F33" s="11" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n"/>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>{{R24}}</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>{{DES24}}</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>{{U24}}</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>{{Q24}}</t>
+        </is>
+      </c>
       <c r="E34" s="11" t="n"/>
       <c r="F34" s="11" t="n"/>
     </row>

</xml_diff>